<commit_message>
data for multiple plot in one figure
</commit_message>
<xml_diff>
--- a/sensitivity_analysis/sensitivity_analysis_parameters.xlsx
+++ b/sensitivity_analysis/sensitivity_analysis_parameters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10824"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucacasamassima/Programming/4th_gen_dh/sensitivity_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7254376-7A58-7B49-9143-CE88021B5921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A93ED18-5208-4944-B518-C58BC8519CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30240" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>n_steps</t>
   </si>
@@ -34,27 +34,6 @@
   </si>
   <si>
     <t>max_val</t>
-  </si>
-  <si>
-    <t>supply_temperature</t>
-  </si>
-  <si>
-    <t>approach_temperature</t>
-  </si>
-  <si>
-    <t>electricity_price</t>
-  </si>
-  <si>
-    <t>gas_price</t>
-  </si>
-  <si>
-    <t>max_cop</t>
-  </si>
-  <si>
-    <t>ir</t>
-  </si>
-  <si>
-    <t>inv_cost_multiplier</t>
   </si>
   <si>
     <t>num_analysis</t>
@@ -381,7 +360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.1640625" bestFit="1" customWidth="1"/>
@@ -390,10 +369,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -407,137 +386,18 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C2">
         <v>20</v>
       </c>
       <c r="D2">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="E2">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>10</v>
-      </c>
-      <c r="D4">
-        <v>0.5</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5">
-        <v>10</v>
-      </c>
-      <c r="D5">
-        <v>0.5</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6">
-        <v>20</v>
-      </c>
-      <c r="D6">
-        <v>1.5</v>
-      </c>
-      <c r="E6">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7">
-        <v>10</v>
-      </c>
-      <c r="D7">
-        <v>70</v>
-      </c>
-      <c r="E7">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8">
-        <v>10</v>
-      </c>
-      <c r="D8">
-        <v>0.5</v>
-      </c>
-      <c r="E8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9">
-        <v>20</v>
-      </c>
-      <c r="D9">
-        <v>0.1</v>
-      </c>
-      <c r="E9">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update results after VAT removal and LCOH fix
</commit_message>
<xml_diff>
--- a/sensitivity_analysis/sensitivity_analysis_parameters.xlsx
+++ b/sensitivity_analysis/sensitivity_analysis_parameters.xlsx
@@ -1,24 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucacasamassima/Programming/4th_gen_dh/sensitivity_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A93ED18-5208-4944-B518-C58BC8519CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C18F51B-5114-0F42-88EA-40B47850A0F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30240" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>

</xml_diff>